<commit_message>
two decimal points for height, weight, output
</commit_message>
<xml_diff>
--- a/report/bocfp.xlsx
+++ b/report/bocfp.xlsx
@@ -35,7 +35,7 @@
     <t>Relationship</t>
   </si>
   <si>
-    <t>Mark aaron</t>
+    <t>Mark Aaron</t>
   </si>
   <si>
     <t>Acupiado</t>
@@ -44,7 +44,7 @@
     <t>Rachell</t>
   </si>
   <si>
-    <t>P12</t>
+    <t>P12C955</t>
   </si>
   <si>
     <t>Mother</t>
@@ -62,13 +62,13 @@
     <t>Velasco</t>
   </si>
   <si>
-    <t>P11086</t>
+    <t>P1108Q5</t>
   </si>
   <si>
     <t>Guardian</t>
   </si>
   <si>
-    <t>Francin kate</t>
+    <t>Francin Kate</t>
   </si>
   <si>
     <t>Hallarde</t>
@@ -80,7 +80,7 @@
     <t>Lara</t>
   </si>
   <si>
-    <t>P6</t>
+    <t>P696S25</t>
   </si>
   <si>
     <t>Height</t>
@@ -102,6 +102,30 @@
   </si>
   <si>
     <t>User Last Name</t>
+  </si>
+  <si>
+    <t>Underweight</t>
+  </si>
+  <si>
+    <t>May 03, 2023 04:21 PM</t>
+  </si>
+  <si>
+    <t>Jenny</t>
+  </si>
+  <si>
+    <t>De Leon</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>May 03, 2023 04:23 PM</t>
+  </si>
+  <si>
+    <t>Overweight</t>
+  </si>
+  <si>
+    <t>May 03, 2023 05:28 PM</t>
   </si>
 </sst>
 </file>
@@ -290,6 +314,102 @@
         <v>29</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2">
+        <v>11</v>
+      </c>
+      <c r="D2">
+        <v>135.1</v>
+      </c>
+      <c r="E2">
+        <v>29.4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2">
+        <v>16.11</v>
+      </c>
+      <c r="H2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <v>129.3</v>
+      </c>
+      <c r="E3">
+        <v>35.5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3">
+        <v>21.23</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4">
+        <v>7</v>
+      </c>
+      <c r="D4">
+        <v>120.9</v>
+      </c>
+      <c r="E4">
+        <v>39.3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4">
+        <v>26.89</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added purok on child list sheet
</commit_message>
<xml_diff>
--- a/report/bocfp.xlsx
+++ b/report/bocfp.xlsx
@@ -33,6 +33,9 @@
   </si>
   <si>
     <t>Relationship</t>
+  </si>
+  <si>
+    <t>Purok</t>
   </si>
   <si>
     <t>Mark Aaron</t>
@@ -191,74 +194,86 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2">
         <v>11</v>
       </c>
       <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
       <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2">
         <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3">
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -287,30 +302,30 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2">
         <v>11</v>
@@ -322,24 +337,24 @@
         <v>29.4</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G2">
         <v>16.11</v>
       </c>
       <c r="H2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3">
         <v>8</v>
@@ -351,24 +366,24 @@
         <v>35.5</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3">
         <v>21.23</v>
       </c>
       <c r="H3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -380,16 +395,16 @@
         <v>39.3</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4">
         <v>26.89</v>
       </c>
       <c r="H4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working on range for generate report
</commit_message>
<xml_diff>
--- a/report/bocfp.xlsx
+++ b/report/bocfp.xlsx
@@ -38,7 +38,7 @@
     <t>Purok</t>
   </si>
   <si>
-    <t>Mark Aaron</t>
+    <t>Mark aaron</t>
   </si>
   <si>
     <t>Acupiado</t>
@@ -47,7 +47,7 @@
     <t>Rachell</t>
   </si>
   <si>
-    <t>P12C955</t>
+    <t>P1235S5</t>
   </si>
   <si>
     <t>Mother</t>
@@ -65,13 +65,13 @@
     <t>Velasco</t>
   </si>
   <si>
-    <t>P1108Q5</t>
+    <t>P11086</t>
   </si>
   <si>
     <t>Guardian</t>
   </si>
   <si>
-    <t>Francin Kate</t>
+    <t>Francin kate</t>
   </si>
   <si>
     <t>Hallarde</t>
@@ -83,7 +83,7 @@
     <t>Lara</t>
   </si>
   <si>
-    <t>P696S25</t>
+    <t>P665V65</t>
   </si>
   <si>
     <t>Height</t>
@@ -104,25 +104,22 @@
     <t>Recorded By</t>
   </si>
   <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Jan 27, 2022 01:31 PM</t>
+  </si>
+  <si>
+    <t>Jenny De leon</t>
+  </si>
+  <si>
     <t>Underweight</t>
   </si>
   <si>
-    <t>May 03, 2023 04:21 PM</t>
-  </si>
-  <si>
-    <t>Jenny De Leon</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>May 03, 2023 04:23 PM</t>
-  </si>
-  <si>
-    <t>Overweight</t>
-  </si>
-  <si>
-    <t>May 03, 2023 05:28 PM</t>
+    <t>Mar 27, 2023 04:23 PM</t>
+  </si>
+  <si>
+    <t>Mar 27, 2023 04:24 PM</t>
   </si>
 </sst>
 </file>
@@ -221,7 +218,7 @@
         <v>12</v>
       </c>
       <c r="H2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -247,7 +244,7 @@
         <v>18</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -273,7 +270,7 @@
         <v>18</v>
       </c>
       <c r="H4">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -331,16 +328,16 @@
         <v>11</v>
       </c>
       <c r="D2">
-        <v>135.1</v>
+        <v>132</v>
       </c>
       <c r="E2">
-        <v>29.4</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
         <v>30</v>
       </c>
       <c r="G2">
-        <v>16.11</v>
+        <v>19.51</v>
       </c>
       <c r="H2" t="s">
         <v>31</v>
@@ -360,16 +357,16 @@
         <v>8</v>
       </c>
       <c r="D3">
-        <v>129.3</v>
+        <v>122</v>
       </c>
       <c r="E3">
-        <v>35.5</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
         <v>33</v>
       </c>
       <c r="G3">
-        <v>21.23</v>
+        <v>16.12</v>
       </c>
       <c r="H3" t="s">
         <v>34</v>
@@ -389,19 +386,19 @@
         <v>7</v>
       </c>
       <c r="D4">
-        <v>120.9</v>
+        <v>120</v>
       </c>
       <c r="E4">
-        <v>39.3</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4">
+        <v>13.89</v>
+      </c>
+      <c r="H4" t="s">
         <v>35</v>
-      </c>
-      <c r="G4">
-        <v>26.89</v>
-      </c>
-      <c r="H4" t="s">
-        <v>36</v>
       </c>
       <c r="I4" t="s">
         <v>32</v>

</xml_diff>